<commit_message>
Will update pest reports in a bit
</commit_message>
<xml_diff>
--- a/pest_report_text.xlsx
+++ b/pest_report_text.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxin\Documents\DDRP_pest_trends\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6502F3-C22F-4872-83C4-6CBAB4EC603E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE0D0FD-34CC-4DAE-A7C9-FEAD63E758D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B23C547D-801B-4841-A1A2-09C2209AF13E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>pest_name</t>
   </si>
@@ -158,237 +158,71 @@
     <t>Tuta absoluta</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Native to Japan, the Japanese beetle (JPB), </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Popillia japonica </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Newman (Coleoptera: Scarabaeidae), is a highly polyphagous pest with more than 400 host plants, including food crops, fruit trees, turfgrass, and ornamental plants (Fleming 1972,  EPPO 2020, Tayeh et al. 2023). Since its first U.S. detection in 1916 in New Jersey, the beetle has become widespread throughout the eastern and central U.S. as well as parts of eastern Canada (Dickerson and Weiss 1918, Fleming 1972, EPPO 2020, Althoff and Rice 2022). Outbreaks in Colorado and California were eradicated (Althoff and Rice 2022); however, JPB is established in a small number of locations in the Pacific Northwest, including in British Columbia, Washington, and Oregon (EPPO 2020, Stoven et al. 2021, Zhu et al. 2023). The pest is also present in parts of Europe and eastern Russia and has been reported in India (India Biodiversity Portal 2016, EPPO 2020).</t>
-    </r>
-  </si>
-  <si>
-    <t>The beetle is univoltine or semivoltine (2-year life cycle) depending on local climatic conditions (Fleming 1972, Vittum 1986, EPPO 2020). Larvae overwinter as second or third instars in the soil, typically beneath managed turfgrass areas like lawns, pasture, and golf courses. Total associated costs of JPB in the U.S. are estimated at $460 million annually, with $234 million a year spent on control and turf replacement costs (Fleming 1972, USDA-APHIS 2015). </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The spotted lanternfly (SLF), </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lycorma delicatula</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (White) (Hemiptera: Fulgoridae), is a highly polyphagous planthopper that feeds on a wide variety of agricultural and nonagricultural plants, including grape vines, fruit and walnut trees, as well as ornamental trees (Chu 1930, Barringer and Ciafré 2020, EPPO 2021). SLF adults damage plants directly by feeding on plant sap, and  sooty mold caused by excrement can impede photosynthesis and attract additional pests (Dara et al. 2015, Urban and Leach 2023).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Native to China, SLF was first detected in the U.S. in 2014 in Pennsylvania and has since spread to at least 20 eastern states (Urban and Leach 2023, NYSIPM 2025). Over the past 20 years, it has also become a major pest in South Korea (Han et al. 2008). Introduced populations of tree-of-heaven [</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Ailanthus altissima </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(Mill.) Swingle], SLF’s preferred host plant, has facilitated the invasion of the pest (Barringer and Ciafré 2020). In suburban landscapes, SLF can become a nuisance as thousands of adults may swarm on trees (Urban and Leach 2023). </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Native to Australia, the light brown apple moth (LBAM), </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Epiphyas postvittana</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (Walker) (Lepidoptera: Tortricidae), is invasive in the United States, the United Kingdom, New Zealand, New Caledonia, and the Azores, with multiple interceptions reported in other countries (Danthanarayana 1975, EPPO 2024, Zhang et al. 2024). The highly polyphagous pest has over 500 reported host plants, though its economic impacts have been greatest for apple, pears, and grapes (Brinkerhoff 2011).</t>
-    </r>
-  </si>
-  <si>
-    <t>Due to a lack of diapause or other synchronizing factors, such as photoperiod or temperature, LBAM exhibits overlapping generations (Sullivan et al. 2014, Buergi et al. 2011). LBAM infestation can result in market access issues due to the risks of transporting live larvae on a large variety of host plants (Suckling et al. 2014). The pests’s distribution in the U.S. is limited to Hawaii, where it was first reported in 1893, and in California, where it was first confirmed in 2007 and now persists mainly around San Francisco and along the coast (Zimmerman 1978, Suckling and Brockerhoff 2010, Barker et al. 2020).</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The emerald ash borer (EAB), </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Agrilus planipennis </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Fairmaire (Coleoptera: Buprestidae), is a flat-headed, wood-boring beetle native to eastern Asia that almost exclusively requires ash trees (</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Fraxinus</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> spp.) to complete its life cycle (Poland et al. 2015, USDA 2025). It was first discovered in North America in 2002 in Michigan and Ontario, though it likely had entered Michigan in the early to mid-1990s (Siegert et al. 2014). EAB is now present in 37 U.S. states and six Canadian provinces (EPPO 2025, USDA-APHIS 2025). Upon hatching, eggs laid by adult beetles in ash bark crevices burrow into the tree to feed on the inner phloem, outer xylem, and cambium, where young larvae or pre-pupae overwinter in serpentine larval galleries (Tluczek et al. 2011, Poland et al. 2015). This feeding usually results in the death of the tree within about six years (Knight et al. 2013). EAB’s cryptic nature, in which all life stages except for the adult beetle are inside of trees, makes early detection of this pest extremely difficult (Haack et al. 2002, USDA-APHIS 2025). </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>All North American ash species are vulnerable to EAB, though blue ash (</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>F. quadrangulata</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Michaux) appears to be less preferred (Poland et al. 2015). In its native range, EAB generally attacks trees that are already stressed (reviewed by Tluczek et al. 2011). In North America, it attacks both healthy and stressed trees, though stressed trees produce higher numbers of adults (Poland and McCullough 2006, Tluczek et al. 2011). White fringetree [</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Chionanthus virginicus</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> L. (Oleaceae)], and olive [</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Olea europaea </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">L. (Oleaceae)], both of which are in the same family as </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Fraxinus </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>spp., are possible hosts for EAB; however, insects may exhibit higher mortality rates on these species (Rutledge and Arango-Velez 2017, Peterson and Cipollini 2020). The financial impact of EAB in the U.S. is estimated to be in the billions of dollars (Aukema et al. 2011). Additionally, the widespread loss of ash trees has resulted in decreased biodiversity and lost ecosystem services (Schrader et al. 2021).</t>
-    </r>
+    <t>The Asian longhorned beetle (ALB), Anoplophora glabripennis Motschulsky (Coleoptera: Cerambycidae), is a xylophagous pest native to the Korean peninsula and eastern China. In the United States, the beetle was first discovered on Long Island, NY, in 1996, where it likely arrived via wood packaging from China. The pest spread to several sites in the eastern United States and Canada but has since been eradicated in Illinois, New Jersey, New York City, Boston, Mississauga, and Toronto. However, infestations currently persist in central Long Island, NY; Worcester County, MA; Clermont County, OH; and Charleston County, SC. ALB is a major threat to the maple hardwood lumber and sugar maple syrup industries, as well as tourism associated with fall colors in maple trees. The cost of a complete infestation of all urban areas in the United States has been estimated at $669 billion.</t>
+  </si>
+  <si>
+    <t>The Asiatic rice borer (ASRB), Chilo suppressalis Walker (Lepidoptera: Crambiidae), is a stem borer and major pest of rice and other grasses, including water oat, sorghum, millet, and corn throughout Asia, Oceana, the Middle East, and Europe. ASRB larvae cause major damage to rice crops by severing panicles or the vascular system of tillers leading to white earheads and dead heart. Larvae can cause substantial economic losses, with reports of 20% yield loss in some scenarios. The pest is present in Hawaii and is frequently intercepted at United States ports.</t>
+  </si>
+  <si>
+    <t>Native to the Mediterranean region, the honeydew moth, Cryptoblabes gnidiella (Lepidoptera: Pyralidae), is a highly polyphagous pest that can act as both a primary and secondary pest of numerous economically important crops, including avocado, citrus, corn, cotton, grape, loquat, pomegranate, rice, and wheat. It is commonly associated with coccoids and pseudococcids, which produce honeydew that serves as a food source for its larvae, although it can also directly damage the fruit of certain host plants. CGN has spread widely across southern Europe, parts of Africa, and several regions worldwide, including Brazil, Fiji, India, Malaysia, New Zealand, Uruguay, and Hawaii in the United States. Although it has not been established in the contiguous United States, it has been intercepted frequently at ports of entry, often originating from countries where its establishment has not been documented.</t>
+  </si>
+  <si>
+    <t>The emerald ash borer (EAB), Agrilus planipennis Fairmaire (Coleoptera: Buprestidae), is a flat-headed, wood-boring beetle native to eastern Asia that relies almost exclusively on ash trees (Fraxinus spp.) to complete its life cycle. It was first detected in North America in 2002 in Michigan and Ontario, although it likely arrived in Michigan during the early to mid-1990s. EAB is now present in 37 U.S. states and six Canadian provinces. Adult beetles lay eggs in bark crevices, and upon hatching, larvae burrow into the tree to feed on the inner phloem, outer xylem, and cambium. They overwinter as larvae or pre-pupae within characteristic serpentine galleries beneath the bark. This feeding disrupts the tree’s ability to transport water and nutrients, typically leading to tree death within several years. EAB’s cryptic nature, in which all life stages except for the adult beetle are inside of trees, makes early detection of this pest extremely difficult.</t>
+  </si>
+  <si>
+    <t>All North American ash species are susceptible to emerald ash borer, although blue ash (F. quadrangulata Michaux) appears to be less preferred. In its native range, the beetle primarily infests stressed or weakened trees, whereas in North America it readily attacks both healthy and stressed individuals, with stressed trees often supporting higher beetle densities. Other members of the olive family, such as white fringetree (Chionanthus virginicus L.) and olive (Olea europaea L.), may also serve as hosts, though survival rates on these species appear to be lower. The economic impact of EAB in the United States has reached billions of dollars, and the widespread loss of ash trees has led to reduced biodiversity and the degradation of important ecosystem services.</t>
+  </si>
+  <si>
+    <t>The Egyptian cottonworm (ECW), Spodoptera littoralis Boisduval (Lepidoptera: Noctuidae), is a highly destructive and polyphagous moth distributed across southern Europe, the Mediterranean basin, the Middle East, Africa, China, and India. With a host range spanning more than 80 plant species in over 40 families, it is a major pest of crops such as cotton, maize, potato, sugarcane, soybeans, vegetables, and wheat. Its development time and survival vary depending on the host plant. The larval stage, which consists of six instars, causes significant damage through extensive defoliation, as well as by attacking growing points and mining or cutting stems. Although ECW is not established in the United States, it has been intercepted multiple times at ports of entry.</t>
+  </si>
+  <si>
+    <t>Native to sub-Saharan Africa, the false codling moth, Thaumatotibia leucotreta Meyrick (Lepidoptera: Tortricidae), is a highly polyphagous pest now distributed throughout much of Africa and parts of the Middle East, including Israel. It infests a wide range of economically important crops, including avocado, citrus, corn, cotton, eggplant, grapes, stone fruits, peppers, and cut roses. The species undergoes five larval instars, during which larvae bore into fruit, causing direct damage before exiting to form cocoons in the soil. In 2008, a single adult male was detected in the wild in California and was successfully eradicated. Although the pest is not established in the United States, it has been repeatedly intercepted at ports of entry in both cargo and passenger baggage. If it were to establish, it could lead to substantial economic losses, potentially reaching billions of dollars.</t>
+  </si>
+  <si>
+    <t>Native to Japan, the Japanese beetle (JPB), Popillia japonica Newman (Coleoptera: Scarabaeidae), is a highly polyphagous pest with a host range exceeding 400 plant species, including food crops, fruit trees, turfgrass, and ornamental plant. Since its initial detection in the United States in 1916 in New Jersey, it has spread widely across the eastern and central regions of the country, as well as parts of eastern Canada. Although isolated infestations have been successfully eradicated in several western states, including Colorado, Nevada, and California, the beetle persists in localized areas of the Pacific Northwest, including parts of British Columbia, Washington, and Oregon. Total associated costs of JPB in the United States are estimated at $460 million annually, with $234 million a year spent on control and turf replacement costs.</t>
+  </si>
+  <si>
+    <t>Native to Australia, the light brown apple moth (LBAM), Epiphyas postvittana (Walker) (Lepidoptera: Tortricidae), is an invasive species established in the United States, the United Kingdom, New Zealand, New Caledonia, and the Azores, with additional interceptions reported worldwide. This highly polyphagous pest has a host range exceeding 500 plant species, although its most significant economic impacts have been observed in apples, pears, and grapes. Infestations can create market access challenges due to the risk of transporting live larvae on a wide variety of host plants. In the United States, its distribution is currently limited to Hawaii, where it was first reported in 1893, and California, where it was confirmed in 2007 and now persists primarily in the San Francisco Bay Area, the Central Coast, and parts of southern California.</t>
+  </si>
+  <si>
+    <t>The oak ambrosia beetle (OAB), Platypus quercivorus Murayama (Coleoptera: Platypodidae), is a destructive forest pest and vector of its symbiotic fungal pathogen, Raffaelea quercivora Kubono &amp; Shin-Ito. This fungus causes Japanese oak wilt disease (JOW), which kills both healthy and stressed trees by disrupting tracheary function. Suitable host plants for reproduction include species of Quercus as well as other members of the Fagaceae family, such as chestnut (Castanea spp.), chinquapin (Castanopsis spp.), and stone oaks (Lithocarpus spp.). However, OAB may also attack non-host tree species located near areas experiencing mass infestation.</t>
+  </si>
+  <si>
+    <t>Females construct galleries and inoculate them with the symbiotic fungus prior to oviposition, producing larvae that feed on the fungal growth. OAB is distributed across India, Indonesia, Japan, and Papua New Guinea; however, R. quercivora has only been reported in Japan, where the beetle–fungus complex has caused extensive oak mortality. The beetle shows a preference for larger trees due to their higher water content, making abandoned oak coppice forests in Japan particularly vulnerable to infestation. If introduced to the United States, OAB and JOW could result in substantial economic, environmental, and social impacts.</t>
+  </si>
+  <si>
+    <t>The Japanese pine sawyer beetle (JPSB), Monochamus alternatus Hope (Coleoptera: Cerambycidae), is a major vector of nematodes that cause pine wilt disease. Native to East Asia, including mainland China, Taiwan, Laos, Korea, and Japan, it has expanded its range to additional parts of Asia, including Vietnam. Adult beetles carry and transmit nematodes—most notably Bursaphelenchus xylophilus—while feeding on healthy pine trees. Infection leads to blockage of the xylem, with visible symptoms often developing within a few weeks. Females lay eggs in weakened or diseased trees, where larvae develop beneath the bark and later overwinter as fourth- or fifth-instar larvae within the xylem or sapwood. Prior to adult emergence, nematodes associate with newly formed beetles, allowing the transmission cycle to continue. Although B. xylophilus is native to North America and typically causes little damage in its native range, the beetle is also capable of vectoring other nematode species not present in North America. In regions where pine wilt disease has been introduced, such as parts of Europe and Asia, it has caused substantial economic losses in forest systems. Host plants of the Japanese pine sawyer beetle are primarily conifers, particularly species within the genera Pinus, Abies, Picea, Larix, and Cedrus, although some hardwood genera, such as Malus and Acer, may also serve as occasional hosts.</t>
+  </si>
+  <si>
+    <t>The Old World bollworm (OWBW), Helicoverpa armigera (Hübner) (Lepidoptera: Noctuidae), is a highly polyphagous pest that feeds on agricultural crops from 68 plant families, including chickpea, corn, cotton, tobacco, tomato, potato, and soybean. It is widely distributed across much of Europe, Asia, Africa, and Australasia, and began expanding into Central and South America in 2013. In 2015, several specimens were detected in Florida, although populations did not become established. The species is capable of long-distance migration, traveling up to 2,000 km when assisted by favorable winds. It has also developed resistance to multiple insecticides and some transgenic crops. If established in the United States, OWBW could place crops valued at an estimated $78 billion annually at risk of damage.</t>
+  </si>
+  <si>
+    <t>The pine-tree lappet moth (PTLM), Dendrolimus pini Linnaeus (Lepidoptera: Lasiocampidae), is an economically important defoliator of pine trees native to Europe and Asia. Its current distribution spans much of Europe, Russia, Kazakhstan, northern China, and Morocco. The species primarily feeds on Scots pine (Pinus sylvestris), but it can also develop successfully on at least 17 other pine species, as well as Douglas-fir (Pseudotsuga menziesii) and eastern hemlock (Tsuga canadensis), and may be capable of establishing on additional Pinus species outside its current range. Trees that survive defoliation often require several years to recover and may become more susceptible to secondary pests. If introduced to the United States, PTLM could cause substantial damage to pine-dominated forests and monoculture plantations, with potentially significant economic impacts on the timber and Christmas tree industries.</t>
+  </si>
+  <si>
+    <t>The spotted lanternfly (SLF), Lycorma delicatula (White) (Hemiptera: Fulgoridae), is a highly polyphagous planthopper that feeds on a broad range of agricultural and non-agricultural plants, including grapevines, fruit and nut trees, and ornamental species. Adults cause direct damage by feeding on plant sap, while the accumulation of honeydew promotes the growth of sooty mold, which can inhibit photosynthesis and attract additional pests. Native to China, SLF was first detected in the United States in 2014 in Pennsylvania and has since spread to at least 20 eastern states. The widespread presence of its preferred host, tree-of-heaven (Ailanthus altissima (Mill.) Swingle), has facilitated its rapid expansion. In suburban and urban environments, SLF can become a significant nuisance, with large aggregations of adults often swarming on trees. The species has already caused substantial economic impacts, including estimated annual losses of $8.8 million to New York’s grape industry alone.</t>
+  </si>
+  <si>
+    <t>The common or cotton cutworm (SLI), Spodoptera litura (Fabricius, 1775) (Lepidoptera: Noctuidae), is a highly polyphagous pest that feeds on at least 120 plant species, including economically important crops such as corn, cotton, groundnut, potato, soybean, sweet potato, tea, tobacco, and a wide range of vegetables. Females lay eggs on host plants, and within a few days, emerging larvae begin feeding on plant tissue, causing extensive damage that can lead to stunted growth and reduced marketability. Native to Southeast Asia, SLI is now distributed across Australia, Oceania, several African islands, Hawaii, and other regions of Asia. The pest has been present in Hawaii since 1964 and has been intercepted hundreds of times at U.S. ports of entry, primarily through cargo and passenger baggage. The species has developed resistance to numerous insecticides and transgenic Bt cotton and is capable of long-distance migration, potentially aided by typhoons. Severe defoliation caused by larval feeding has led to significant crop damage and economic losses in affected regions.</t>
+  </si>
+  <si>
+    <t>Widespread across Europe, northern Africa, and Asia, the silver Y moth (SLYM), Autographa gamma Linnaeus (Lepidoptera: Noctuidae), is a highly polyphagous defoliator of cereals, Brassica spp., legumes, tobacco, and a wide range of fruit and vegetable crops, with particularly significant impacts on sugar beet. Adults undertake annual migrations to northern breeding regions across Eurasia to avoid the hot, dry conditions of Mediterranean overwintering areas. Population outbreaks in these breeding regions occur sporadically and are often associated with periods of unusually wet weather. The species is considered a high-risk invasive agricultural pest for the United States, with the potential to damage more than 200 plant species, including lettuce, cabbage, and grape. It has been intercepted hundreds of times at U.S. ports of entry on approximately 130 plant taxa and is considered to have a high likelihood of establishment if introduced.</t>
+  </si>
+  <si>
+    <t>The small tomato borer (STB), Neoleucinodes elegantalis (Guenée) (Lepidoptera: Pyralidae), is an oligophagous pest of Solanum species, including tomato, eggplant, red and green pepper, lulo (naranjilla), and wild Solanum spp. Native to South America, it has expanded its range into Mexico, Central America, and the Caribbean. The species occupies a wide range of climatic conditions in South America, although its distribution varies depending on host plant availability and altitude. Larvae develop through five instars, with the third through fifth instars responsible for most of the fruit damage, and development rates that may vary by host plant. Infestations can result in severe economic losses, with reported yield reductions in South American tomato crops ranging from 45% to 90%. If introduced to the United States, regions with high levels of tomato and pepper production would be particularly vulnerable. In addition, STB poses a significant barrier to the export of solanaceous crops from South America to the United States and the European Union. The pest has been intercepted hundreds of times at U.S. ports of entry, with most interceptions originating from Brazil.</t>
+  </si>
+  <si>
+    <t>The Sunn pest (SUNP), Eurygaster integriceps Puton, 1881 (Hemiptera: Scutelleridae), is a serious and economically important pest of wheat, barley, oats, rye, and sorghum. Its geographic range spans latitudes 25° to 55° N across Eurasia, including much of Eastern Europe, West Asia, Central Asia, and North Africa. Both larvae and adults damage host plants by causing plant death, arresting grain development, or degrading the gluten content of surviving wheat kernels. As a result, flour produced from infested grain yields bread of poor quality and reduced digestibility. In the absence of effective control measures, infestations can lead to complete crop loss. If introduced to the United States, SUNP could cause substantial economic damage to wheat and barley production, which were valued at $7.9 billion and $685 million, respectively, in 2017. Areas at most risk for establishment of SUNP based on host presence are in the Midwestern United States, the Columbia River valley, and the lower Mississippi River valley.</t>
+  </si>
+  <si>
+    <t>The tomato leaf miner (TABS), Phthorimaea absoluta (Meyrick) (formerly Tuta absoluta) (Lepidoptera: Gelechiidae), is a highly destructive pest of tomato and other solanaceous crops, native to Peru. It is now widely distributed across Central and South America and has invaded much of Europe, Africa, and Asia, reaching as far as South Korea. In China, the species has demonstrated an exceptionally rapid spread, with a median dispersal rate exceeding 1,000 km per day. In cooler regions, TABS can persist in protected environments such as greenhouses. Early infestations are difficult to detect, and if left unmanaged, the pest can cause complete crop loss. Its rapid global expansion has led to increased reliance on synthetic insecticides, with associated environmental and health concerns. Climate suitability models indicate that major tomato-producing countries, including the United States, Mexico, and Canada, are at high risk of invasion, which could lead to increased tomato prices.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -399,15 +233,9 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -430,11 +258,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -773,192 +605,232 @@
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="23.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="15.46484375" customWidth="1"/>
+    <col min="1" max="1" width="23.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.53125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.46484375" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="1"/>
-    </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="C4" s="2" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="1" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-    </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="C9" s="3" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>45</v>
-      </c>
+      <c r="C10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="C11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="C12" s="2" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>33</v>
       </c>
+      <c r="C13" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="4"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="C14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="3"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="C15" s="2" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
+      <c r="C16" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
+      <c r="C17" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
+      <c r="C18" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>39</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>